<commit_message>
Fix database mixLength decode to accurately show true durations and clean localStorage cache
</commit_message>
<xml_diff>
--- a/MusicMarshall_Complete_Database.xlsx
+++ b/MusicMarshall_Complete_Database.xlsx
@@ -555,12 +555,12 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>404:29</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>404.49</t>
+          <t>19.50</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -605,12 +605,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>445:27</t>
+          <t>55:30</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>445.45</t>
+          <t>55.50</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -655,12 +655,12 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>87:03</t>
+          <t>28:30</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>87.05</t>
+          <t>28.50</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -705,12 +705,12 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>230:24</t>
+          <t>26:30</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>230.41</t>
+          <t>26.50</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -755,12 +755,12 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>296:58</t>
+          <t>1:41:00</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>296.97</t>
+          <t>101.00</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -805,12 +805,12 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>340:29</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>340.49</t>
+          <t>19.25</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>337:55</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>337.93</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -905,12 +905,12 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>261:07</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>261.13</t>
+          <t>21.50</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>87:03</t>
+          <t>28:30</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>87.05</t>
+          <t>28.50</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1005,12 +1005,12 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>133:07</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>133.13</t>
+          <t>21.00</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1055,12 +1055,12 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>133:07</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>133.13</t>
+          <t>21.00</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>133:07</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>133.13</t>
+          <t>21.00</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1155,12 +1155,12 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>358:24</t>
+          <t>27:00</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>358.41</t>
+          <t>27.00</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>296:58</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>296.97</t>
+          <t>11.40</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1255,12 +1255,12 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>368:39</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>368.65</t>
+          <t>4.00</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1305,12 +1305,12 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>496:39</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>496.65</t>
+          <t>4.50</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>368:39</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>368.65</t>
+          <t>4.00</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1405,12 +1405,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>368:39</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>368.65</t>
+          <t>4.00</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1455,12 +1455,12 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>368:39</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>368.65</t>
+          <t>4.00</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1505,12 +1505,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>506:53</t>
+          <t>45:30</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>506.89</t>
+          <t>45.50</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1555,12 +1555,12 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>112:39</t>
+          <t>3:15:00</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>112.65</t>
+          <t>195.00</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1605,12 +1605,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>286:43</t>
+          <t>1:00:00</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>286.73</t>
+          <t>60.00</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1655,12 +1655,12 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>591:22</t>
+          <t>04:52</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>591.37</t>
+          <t>4.87</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1705,12 +1705,12 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>471:03</t>
+          <t>30:00</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>471.05</t>
+          <t>30.00</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1755,12 +1755,12 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>368:39</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>368.65</t>
+          <t>4.00</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1805,12 +1805,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>634:53</t>
+          <t>46:00</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>634.89</t>
+          <t>46.00</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>284:10</t>
+          <t>03:40</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>284.17</t>
+          <t>3.67</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1905,12 +1905,12 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>560:39</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>560.65</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>112:39</t>
+          <t>03:00</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>112.65</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2005,12 +2005,12 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>112:39</t>
+          <t>03:00</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>112.65</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2055,12 +2055,12 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>424:58</t>
+          <t>04:13</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>424.97</t>
+          <t>4.22</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2105,12 +2105,12 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>79:22</t>
+          <t>02:52</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>79.37</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2155,12 +2155,12 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>232:58</t>
+          <t>03:28</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>232.97</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2205,12 +2205,12 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>296:58</t>
+          <t>03:43</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>296.97</t>
+          <t>3.72</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">

</xml_diff>